<commit_message>
update with new csvs from database errors
</commit_message>
<xml_diff>
--- a/Data for R/DOP/DOP EDI Qry_Presence_Absence Categories to Post.xlsx
+++ b/Data for R/DOP/DOP EDI Qry_Presence_Absence Categories to Post.xlsx
@@ -11725,7 +11725,7 @@
       </c>
       <c r="H123" s="5" t="inlineStr">
         <is>
-          <t>L0493</t>
+          <t>0493</t>
         </is>
       </c>
       <c r="I123" s="5" t="inlineStr">
@@ -11750,9 +11750,15 @@
           <t>0.37</t>
         </is>
       </c>
+      <c r="O123" s="9">
+        <v>18.3</v>
+      </c>
+      <c r="P123" s="9">
+        <v>786</v>
+      </c>
       <c r="Q123" s="9" t="inlineStr">
         <is>
-          <t/>
+          <t>0.37</t>
         </is>
       </c>
       <c r="R123" s="9" t="inlineStr">
@@ -11814,7 +11820,7 @@
       </c>
       <c r="H124" s="5" t="inlineStr">
         <is>
-          <t>L0448</t>
+          <t>448</t>
         </is>
       </c>
       <c r="I124" s="5" t="inlineStr">
@@ -11839,9 +11845,15 @@
           <t>0.06</t>
         </is>
       </c>
+      <c r="O124" s="9">
+        <v>13.9</v>
+      </c>
+      <c r="P124" s="9">
+        <v>137.5</v>
+      </c>
       <c r="Q124" s="9" t="inlineStr">
         <is>
-          <t/>
+          <t>0.06</t>
         </is>
       </c>
       <c r="R124" s="9" t="inlineStr">
@@ -11903,7 +11915,7 @@
       </c>
       <c r="H125" s="5" t="inlineStr">
         <is>
-          <t>L1361</t>
+          <t>1361</t>
         </is>
       </c>
       <c r="I125" s="5" t="inlineStr">
@@ -11925,9 +11937,15 @@
           <t>0.34</t>
         </is>
       </c>
+      <c r="O125" s="9">
+        <v>17.4</v>
+      </c>
+      <c r="P125" s="9">
+        <v>737</v>
+      </c>
       <c r="Q125" s="9" t="inlineStr">
         <is>
-          <t/>
+          <t>0.34</t>
         </is>
       </c>
       <c r="R125" s="9" t="inlineStr">
@@ -11989,7 +12007,7 @@
       </c>
       <c r="H126" s="5" t="inlineStr">
         <is>
-          <t>Vial 1</t>
+          <t>LV1</t>
         </is>
       </c>
       <c r="I126" s="5" t="inlineStr">
@@ -12549,8 +12567,14 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J132" s="8">
+        <v>0.386805555555556</v>
+      </c>
+      <c r="K132" s="9">
+        <v>17.3</v>
+      </c>
       <c r="L132" s="9">
-        <v>8.60000038146973</v>
+        <v>8.600000381</v>
       </c>
       <c r="M132" s="9">
         <v>410</v>
@@ -12567,11 +12591,11 @@
       </c>
       <c r="R132" s="9" t="inlineStr">
         <is>
-          <t/>
+          <t>31</t>
         </is>
       </c>
       <c r="S132" s="9">
-        <v>37.5999984741211</v>
+        <v>37.59999847</v>
       </c>
       <c r="T132" s="9">
         <v>1.2486</v>
@@ -12635,8 +12659,14 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J133" s="8">
+        <v>0.431944444444444</v>
+      </c>
+      <c r="K133" s="9">
+        <v>11.3</v>
+      </c>
       <c r="L133" s="9">
-        <v>10.6000003814697</v>
+        <v>10.60000038</v>
       </c>
       <c r="M133" s="9">
         <v>1113</v>
@@ -12653,7 +12683,7 @@
       </c>
       <c r="R133" s="9" t="inlineStr">
         <is>
-          <t/>
+          <t>131</t>
         </is>
       </c>
       <c r="S133" s="9">
@@ -12721,8 +12751,14 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J134" s="8">
+        <v>0.402083333333333</v>
+      </c>
+      <c r="K134" s="9">
+        <v>9.8</v>
+      </c>
       <c r="L134" s="9">
-        <v>8.80000019073486</v>
+        <v>8.800000191</v>
       </c>
       <c r="M134" s="9">
         <v>541</v>
@@ -12739,11 +12775,11 @@
       </c>
       <c r="R134" s="9" t="inlineStr">
         <is>
-          <t/>
+          <t>34</t>
         </is>
       </c>
       <c r="S134" s="9">
-        <v>38.7999992370605</v>
+        <v>38.79999924</v>
       </c>
       <c r="T134" s="9">
         <v>4.227</v>
@@ -12887,8 +12923,14 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J136" s="8">
+        <v>0.348611111111111</v>
+      </c>
+      <c r="K136" s="9">
+        <v>10.1</v>
+      </c>
       <c r="L136" s="9">
-        <v>9.80000019073486</v>
+        <v>9.800000191</v>
       </c>
       <c r="M136" s="9">
         <v>639</v>
@@ -12909,7 +12951,7 @@
         </is>
       </c>
       <c r="S136" s="9">
-        <v>75.0999984741211</v>
+        <v>75.09999847</v>
       </c>
       <c r="T136" s="9">
         <v>2.5888</v>
@@ -12973,11 +13015,17 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J137" s="8">
+        <v>0.408333333333333</v>
+      </c>
+      <c r="K137" s="9">
+        <v>11.3</v>
+      </c>
       <c r="L137" s="9">
-        <v>9.69999980926514</v>
+        <v>9.699999809</v>
       </c>
       <c r="M137" s="9">
-        <v>232.100006103516</v>
+        <v>232.1000061</v>
       </c>
       <c r="N137" s="9" t="inlineStr">
         <is>
@@ -12995,7 +13043,7 @@
         </is>
       </c>
       <c r="S137" s="9">
-        <v>32.2999992370605</v>
+        <v>32.29999924</v>
       </c>
       <c r="T137" s="9">
         <v>6.6357</v>
@@ -13146,10 +13194,10 @@
         <v>11.1</v>
       </c>
       <c r="L139" s="9">
-        <v>22.1000003814697</v>
+        <v>22.10000038</v>
       </c>
       <c r="M139" s="9">
-        <v>323.600006103516</v>
+        <v>323.6000061</v>
       </c>
       <c r="N139" s="9" t="inlineStr">
         <is>
@@ -13231,8 +13279,14 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J140" s="8">
+        <v>0.431944444444444</v>
+      </c>
+      <c r="K140" s="9">
+        <v>4.7</v>
+      </c>
       <c r="L140" s="9">
-        <v>10.1000003814697</v>
+        <v>10.10000038</v>
       </c>
       <c r="M140" s="9">
         <v>3131</v>
@@ -13253,7 +13307,7 @@
         </is>
       </c>
       <c r="S140" s="9">
-        <v>25.1000003814697</v>
+        <v>25.10000038</v>
       </c>
       <c r="T140" s="9">
         <v>3.6947</v>
@@ -13290,7 +13344,7 @@
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t/>
+          <t>KT</t>
         </is>
       </c>
       <c r="D141" s="6">
@@ -13309,13 +13363,16 @@
       </c>
       <c r="H141" s="5" t="inlineStr">
         <is>
-          <t>0011</t>
+          <t>S-011</t>
         </is>
       </c>
       <c r="I141" s="5" t="inlineStr">
         <is>
           <t>DELSME</t>
         </is>
+      </c>
+      <c r="J141" s="8">
+        <v>0.513888888888889</v>
       </c>
       <c r="N141" s="9" t="inlineStr">
         <is>
@@ -13339,6 +13396,9 @@
         <is>
           <t>Y</t>
         </is>
+      </c>
+      <c r="V141" s="10">
+        <v>68</v>
       </c>
       <c r="W141" s="9">
         <v>0.0296</v>
@@ -13391,8 +13451,14 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J142" s="8">
+        <v>0.51875</v>
+      </c>
+      <c r="K142" s="9">
+        <v>6.8</v>
+      </c>
       <c r="L142" s="9">
-        <v>15.3999996185303</v>
+        <v>15.39999962</v>
       </c>
       <c r="M142" s="9">
         <v>4335</v>
@@ -13413,7 +13479,7 @@
         </is>
       </c>
       <c r="S142" s="9">
-        <v>90.4000015258789</v>
+        <v>90.40000153</v>
       </c>
       <c r="T142" s="9">
         <v>2.694</v>
@@ -13477,6 +13543,12 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J143" s="8">
+        <v>0.465972222222222</v>
+      </c>
+      <c r="K143" s="9">
+        <v>8.8</v>
+      </c>
       <c r="L143" s="9">
         <v>16.5</v>
       </c>
@@ -13499,7 +13571,7 @@
         </is>
       </c>
       <c r="S143" s="9">
-        <v>93.6999969482422</v>
+        <v>93.69999695</v>
       </c>
       <c r="T143" s="9">
         <v>2.7079</v>
@@ -13563,11 +13635,17 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J144" s="8">
+        <v>0.520138888888889</v>
+      </c>
+      <c r="K144" s="9">
+        <v>11</v>
+      </c>
       <c r="L144" s="9">
-        <v>11.1999998092651</v>
+        <v>11.19999981</v>
       </c>
       <c r="M144" s="9">
-        <v>386.799987792969</v>
+        <v>386.7999878</v>
       </c>
       <c r="N144" s="9" t="inlineStr">
         <is>
@@ -13585,7 +13663,7 @@
         </is>
       </c>
       <c r="S144" s="9">
-        <v>25.6000003814697</v>
+        <v>25.60000038</v>
       </c>
       <c r="T144" s="9">
         <v>3.8923</v>
@@ -13649,11 +13727,17 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J145" s="8">
+        <v>0.520138888888889</v>
+      </c>
+      <c r="K145" s="9">
+        <v>11</v>
+      </c>
       <c r="L145" s="9">
-        <v>11.1999998092651</v>
+        <v>11.19999981</v>
       </c>
       <c r="M145" s="9">
-        <v>386.799987792969</v>
+        <v>386.7999878</v>
       </c>
       <c r="N145" s="9" t="inlineStr">
         <is>
@@ -13671,7 +13755,7 @@
         </is>
       </c>
       <c r="S145" s="9">
-        <v>25.6000003814697</v>
+        <v>25.60000038</v>
       </c>
       <c r="T145" s="9">
         <v>1.3369</v>
@@ -13735,11 +13819,17 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J146" s="8">
+        <v>0.520138888888889</v>
+      </c>
+      <c r="K146" s="9">
+        <v>11</v>
+      </c>
       <c r="L146" s="9">
-        <v>11.1999998092651</v>
+        <v>11.19999981</v>
       </c>
       <c r="M146" s="9">
-        <v>386.799987792969</v>
+        <v>386.7999878</v>
       </c>
       <c r="N146" s="9" t="inlineStr">
         <is>
@@ -13757,7 +13847,7 @@
         </is>
       </c>
       <c r="S146" s="9">
-        <v>25.6000003814697</v>
+        <v>25.60000038</v>
       </c>
       <c r="T146" s="9">
         <v>1.8949</v>
@@ -13821,6 +13911,12 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J147" s="8">
+        <v>0.532638888888889</v>
+      </c>
+      <c r="K147" s="9">
+        <v>10.8</v>
+      </c>
       <c r="L147" s="9">
         <v>11</v>
       </c>
@@ -13843,7 +13939,7 @@
         </is>
       </c>
       <c r="S147" s="9">
-        <v>30.1000003814697</v>
+        <v>30.10000038</v>
       </c>
       <c r="T147" s="9">
         <v>1.7369</v>
@@ -13907,11 +14003,17 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J148" s="8">
+        <v>0.428472222222222</v>
+      </c>
+      <c r="K148" s="9">
+        <v>7.6</v>
+      </c>
       <c r="L148" s="9">
-        <v>12.1999998092651</v>
+        <v>12.19999981</v>
       </c>
       <c r="M148" s="9">
-        <v>433.899993896484</v>
+        <v>433.8999939</v>
       </c>
       <c r="N148" s="9" t="inlineStr">
         <is>
@@ -13929,7 +14031,7 @@
         </is>
       </c>
       <c r="S148" s="9">
-        <v>27.2000007629395</v>
+        <v>27.20000076</v>
       </c>
       <c r="T148" s="9">
         <v>2.1016</v>
@@ -13993,11 +14095,17 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J149" s="8">
+        <v>0.428472222222222</v>
+      </c>
+      <c r="K149" s="9">
+        <v>7.6</v>
+      </c>
       <c r="L149" s="9">
-        <v>12.1999998092651</v>
+        <v>12.19999981</v>
       </c>
       <c r="M149" s="9">
-        <v>433.899993896484</v>
+        <v>433.8999939</v>
       </c>
       <c r="N149" s="9" t="inlineStr">
         <is>
@@ -14015,7 +14123,7 @@
         </is>
       </c>
       <c r="S149" s="9">
-        <v>27.2000007629395</v>
+        <v>27.20000076</v>
       </c>
       <c r="T149" s="9">
         <v>1.011</v>
@@ -14079,11 +14187,17 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J150" s="8">
+        <v>0.428472222222222</v>
+      </c>
+      <c r="K150" s="9">
+        <v>7.6</v>
+      </c>
       <c r="L150" s="9">
-        <v>12.1999998092651</v>
+        <v>12.19999981</v>
       </c>
       <c r="M150" s="9">
-        <v>433.899993896484</v>
+        <v>433.8999939</v>
       </c>
       <c r="N150" s="9" t="inlineStr">
         <is>
@@ -14101,7 +14215,7 @@
         </is>
       </c>
       <c r="S150" s="9">
-        <v>27.2000007629395</v>
+        <v>27.20000076</v>
       </c>
       <c r="T150" s="9">
         <v>1.8063</v>
@@ -14168,11 +14282,17 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J151" s="8">
+        <v>0.428472222222222</v>
+      </c>
+      <c r="K151" s="9">
+        <v>7.6</v>
+      </c>
       <c r="L151" s="9">
-        <v>12.1999998092651</v>
+        <v>12.19999981</v>
       </c>
       <c r="M151" s="9">
-        <v>433.899993896484</v>
+        <v>433.8999939</v>
       </c>
       <c r="N151" s="9" t="inlineStr">
         <is>
@@ -14190,7 +14310,7 @@
         </is>
       </c>
       <c r="S151" s="9">
-        <v>27.2000007629395</v>
+        <v>27.20000076</v>
       </c>
       <c r="T151" s="9">
         <v>3.5917</v>
@@ -14257,6 +14377,12 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J152" s="8">
+        <v>0.4</v>
+      </c>
+      <c r="K152" s="9">
+        <v>7.4</v>
+      </c>
       <c r="L152" s="9">
         <v>14.5</v>
       </c>
@@ -14279,7 +14405,7 @@
         </is>
       </c>
       <c r="S152" s="9">
-        <v>26.7000007629395</v>
+        <v>26.70000076</v>
       </c>
       <c r="T152" s="9">
         <v>2.4354</v>
@@ -14344,7 +14470,7 @@
         <v>0.492997685185185</v>
       </c>
       <c r="K153" s="9">
-        <v>26.7</v>
+        <v>8.13816</v>
       </c>
       <c r="L153" s="9">
         <v>16</v>
@@ -14429,8 +14555,14 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J154" s="8">
+        <v>0.527777777777778</v>
+      </c>
+      <c r="K154" s="9">
+        <v>8.4</v>
+      </c>
       <c r="L154" s="9">
-        <v>23.2000007629395</v>
+        <v>23.20000076</v>
       </c>
       <c r="M154" s="9">
         <v>586</v>
@@ -14525,7 +14657,7 @@
         <v>0.406956018518519</v>
       </c>
       <c r="K155" s="9">
-        <v>14.3</v>
+        <v>4.35864</v>
       </c>
       <c r="L155" s="9">
         <v>16.9</v>
@@ -14613,6 +14745,12 @@
           <t>DELSME</t>
         </is>
       </c>
+      <c r="J156" s="8">
+        <v>0.365266203703704</v>
+      </c>
+      <c r="K156" s="9">
+        <v>7.1628</v>
+      </c>
       <c r="L156" s="9">
         <v>15.8</v>
       </c>
@@ -14699,11 +14837,14 @@
       <c r="J157" s="8">
         <v>0.365277777777778</v>
       </c>
+      <c r="K157" s="9">
+        <v>12.1</v>
+      </c>
       <c r="L157" s="9">
-        <v>8.19999980926514</v>
+        <v>8.199999809</v>
       </c>
       <c r="M157" s="9">
-        <v>169.600006103516</v>
+        <v>169.6000061</v>
       </c>
       <c r="N157" s="9" t="inlineStr">
         <is>
@@ -14719,6 +14860,9 @@
         <is>
           <t>14</t>
         </is>
+      </c>
+      <c r="S157" s="9">
+        <v>120</v>
       </c>
       <c r="T157" s="9">
         <v>4.1981</v>
@@ -15191,8 +15335,11 @@
       <c r="J163" s="8">
         <v>0.366666666666667</v>
       </c>
+      <c r="K163" s="9">
+        <v>3.9</v>
+      </c>
       <c r="L163" s="9">
-        <v>18.7999992370605</v>
+        <v>18.79999924</v>
       </c>
       <c r="M163" s="9">
         <v>6651</v>
@@ -15211,6 +15358,9 @@
         <is>
           <t>40</t>
         </is>
+      </c>
+      <c r="S163" s="9">
+        <v>41.5</v>
       </c>
       <c r="T163" s="9">
         <v>0.6435</v>
@@ -15277,8 +15427,11 @@
       <c r="J164" s="8">
         <v>0.461111111111111</v>
       </c>
+      <c r="K164" s="9">
+        <v>6.4</v>
+      </c>
       <c r="L164" s="9">
-        <v>19.6000003814697</v>
+        <v>19.60000038</v>
       </c>
       <c r="M164" s="9">
         <v>9420</v>
@@ -15297,6 +15450,9 @@
         <is>
           <t>31</t>
         </is>
+      </c>
+      <c r="S164" s="9">
+        <v>45.79999924</v>
       </c>
       <c r="T164" s="9">
         <v>2.0226</v>
@@ -15363,11 +15519,14 @@
       <c r="J165" s="8">
         <v>0.3875</v>
       </c>
+      <c r="K165" s="9">
+        <v>17.4</v>
+      </c>
       <c r="L165" s="9">
         <v>8.5</v>
       </c>
       <c r="M165" s="9">
-        <v>242.699996948242</v>
+        <v>242.6999969</v>
       </c>
       <c r="N165" s="9" t="inlineStr">
         <is>
@@ -15383,6 +15542,9 @@
         <is>
           <t>26</t>
         </is>
+      </c>
+      <c r="S165" s="9">
+        <v>47.70000076</v>
       </c>
       <c r="T165" s="9">
         <v>3.1539</v>

</xml_diff>